<commit_message>
Correct seasonality claim in value number (tax forms are onboarding-driven, L171/L201)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016P9Z9B879NzE7WcSVWNcxZ
</commit_message>
<xml_diff>
--- a/Analysis/output/Value number raw data.xlsx
+++ b/Analysis/output/Value number raw data.xlsx
@@ -231,7 +231,7 @@
     <t xml:space="preserve">Tax-form share of Q1 minutes (W-9/W-8 season)</t>
   </si>
   <si>
-    <t xml:space="preserve">Q1 contains tax-form season → annualising Q1 overstates load (conservative)</t>
+    <t xml:space="preserve">NOT a proven peak: tax forms come with new-creator onboarding (slack L171) and Ops calls June 'tax form season again' (L201). Treat as neutral.</t>
   </si>
   <si>
     <t xml:space="preserve">Hours, 2026-01</t>
@@ -2523,7 +2523,7 @@
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>52</v>
       </c>

</xml_diff>